<commit_message>
chore(template): update Excel format template
</commit_message>
<xml_diff>
--- a/Формат_выгрузки.xlsx
+++ b/Формат_выгрузки.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danthecoolest/PycharmProjects/lab_unloading/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danthecoolest/PycharmProjects/lab_parser/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31412BD8-C07B-A04D-AEFF-8265FB89171C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5802AFB3-3B76-9C42-A884-DB2F4D77F94E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="840" windowWidth="30240" windowHeight="17300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>№ п/п</t>
   </si>
@@ -58,23 +58,29 @@
     <t>трихинеллез, отрицательный</t>
   </si>
   <si>
-    <t>ЧЗ005649</t>
-  </si>
-  <si>
     <t>12.03.2025</t>
   </si>
   <si>
-    <t>ОПВК Данковского филиал АО ЧМПЗ</t>
-  </si>
-  <si>
-    <t>179568-181417 от 27.02.2025 г.</t>
+    <t>Хозяйствующий субъект - получатель</t>
+  </si>
+  <si>
+    <t>Предприятие - получатель</t>
+  </si>
+  <si>
+    <t>Акционерное общество "Куриное Царство" (АО "КЦ") (140162, Российская Федерация, Московская обл., Раменский район, с. Константиново, стр. владение 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "ТОРГОВЫЙ ДОМ ЧЕРКИЗОВО", ИНН: </t>
+  </si>
+  <si>
+    <t>хххххх</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -89,6 +95,17 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -126,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -151,6 +168,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -456,19 +479,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="56.1640625" customWidth="1"/>
     <col min="3" max="3" width="167.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="46.5" style="8" customWidth="1"/>
     <col min="5" max="5" width="37.83203125" style="5" customWidth="1"/>
-    <col min="6" max="6" width="157.6640625" style="4" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" style="7" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.5" style="5" customWidth="1"/>
+    <col min="6" max="6" width="85" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="131.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="157.6640625" style="4" customWidth="1"/>
+    <col min="9" max="9" width="16.83203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.5" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -484,17 +509,23 @@
       <c r="E1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -504,23 +535,24 @@
       <c r="C2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" s="5" t="s">
+      <c r="F2" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="H2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="I2" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="J2" s="5" t="s">
         <v>11</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>